<commit_message>
first working copy of robust system with regression and classification model
</commit_message>
<xml_diff>
--- a/data/dataset.xlsx
+++ b/data/dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\TechM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vijay\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB12554-0826-49BA-B9F8-F410677B3C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A6E7C3-7EFA-46BC-945C-2147F94F8BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" tabRatio="319" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="319" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data FY 24-25" sheetId="2" r:id="rId1"/>
@@ -18,10 +18,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Data FY 24-25'!$A$5:$AP$431</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -87,9 +96,6 @@
     <t>TW Iron</t>
   </si>
   <si>
-    <t>RW  Hardness</t>
-  </si>
-  <si>
     <t>RW S Solids</t>
   </si>
   <si>
@@ -102,16 +108,10 @@
     <t>RW Manganese</t>
   </si>
   <si>
-    <t xml:space="preserve">RW Conductivity  </t>
-  </si>
-  <si>
     <t>RW Calcium</t>
   </si>
   <si>
     <t>RW Magnesium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RW Alkalinity </t>
   </si>
   <si>
     <t>RW Ammonia as N</t>
@@ -138,16 +138,10 @@
     <t>TW Manganese</t>
   </si>
   <si>
-    <t xml:space="preserve">TW Conductivity  </t>
-  </si>
-  <si>
     <t>TW Calcium</t>
   </si>
   <si>
     <t>TW Magnesium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TW Alkalinity </t>
   </si>
   <si>
     <t>TW Ammonia as N</t>
@@ -206,6 +200,21 @@
   </si>
   <si>
     <t>Raw Water and Treated Water Analysis - Apr '24 - May '25</t>
+  </si>
+  <si>
+    <t>RW Conductivity</t>
+  </si>
+  <si>
+    <t>TW Conductivity</t>
+  </si>
+  <si>
+    <t>TW Alkalinity</t>
+  </si>
+  <si>
+    <t>RW Alkalinity</t>
+  </si>
+  <si>
+    <t>RW Hardness</t>
   </si>
 </sst>
 </file>
@@ -1061,47 +1070,47 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:AP431"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.85546875" style="38" bestFit="1" customWidth="1"/>
-    <col min="2" max="6" width="10.7109375" style="41" customWidth="1"/>
-    <col min="7" max="7" width="10.42578125" style="7" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.5703125" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.86328125" style="38" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="10.73046875" style="41" customWidth="1"/>
+    <col min="7" max="7" width="10.3984375" style="7" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.86328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.73046875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.1328125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.59765625" customWidth="1"/>
+    <col min="13" max="13" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.59765625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.265625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.59765625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.3984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.1328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="15" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="11.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="15.140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.86328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.59765625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.59765625" style="7" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="11.3984375" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.1328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.1328125" style="7" bestFit="1" customWidth="1"/>
     <col min="31" max="32" width="15" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="9.5703125" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="13.59765625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="8.86328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="9.1328125" bestFit="1" customWidth="1"/>
     <col min="40" max="41" width="9" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="8.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:42" ht="17.649999999999999" x14ac:dyDescent="0.45">
       <c r="A1" s="83" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B1" s="83"/>
       <c r="C1" s="83"/>
@@ -1119,9 +1128,9 @@
       <c r="O1" s="83"/>
       <c r="P1" s="83"/>
     </row>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A2" s="84" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B2" s="84"/>
       <c r="C2" s="84"/>
@@ -1139,9 +1148,9 @@
       <c r="O2" s="84"/>
       <c r="P2" s="84"/>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A3" s="85" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B3" s="85"/>
       <c r="C3" s="85"/>
@@ -1159,24 +1168,24 @@
       <c r="O3" s="85"/>
       <c r="P3" s="85"/>
     </row>
-    <row r="4" spans="1:42" s="58" customFormat="1" ht="58.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" s="58" customFormat="1" ht="58.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="57" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="63" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C4" s="63" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D4" s="63" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E4" s="63" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="F4" s="63" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G4" s="63" t="s">
         <v>15</v>
@@ -1197,114 +1206,114 @@
         <v>18</v>
       </c>
       <c r="M4" s="63" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="63" t="s">
         <v>19</v>
       </c>
-      <c r="N4" s="63" t="s">
+      <c r="P4" s="63" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q4" s="63" t="s">
+        <v>20</v>
+      </c>
+      <c r="R4" s="63" t="s">
+        <v>31</v>
+      </c>
+      <c r="S4" s="63" t="s">
+        <v>21</v>
+      </c>
+      <c r="T4" s="63" t="s">
+        <v>39</v>
+      </c>
+      <c r="U4" s="63" t="s">
+        <v>22</v>
+      </c>
+      <c r="V4" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" s="63" t="s">
+        <v>54</v>
+      </c>
+      <c r="X4" s="63" t="s">
+        <v>55</v>
+      </c>
+      <c r="Y4" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="Z4" s="63" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA4" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="O4" s="63" t="s">
-        <v>20</v>
-      </c>
-      <c r="P4" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q4" s="63" t="s">
-        <v>21</v>
-      </c>
-      <c r="R4" s="63" t="s">
+      <c r="AB4" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="AC4" s="63" t="s">
+        <v>24</v>
+      </c>
+      <c r="AD4" s="63" t="s">
+        <v>24</v>
+      </c>
+      <c r="AE4" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="S4" s="63" t="s">
-        <v>22</v>
-      </c>
-      <c r="T4" s="63" t="s">
-        <v>44</v>
-      </c>
-      <c r="U4" s="63" t="s">
-        <v>23</v>
-      </c>
-      <c r="V4" s="63" t="s">
+      <c r="AF4" s="63" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG4" s="63" t="s">
+        <v>57</v>
+      </c>
+      <c r="AH4" s="63" t="s">
+        <v>56</v>
+      </c>
+      <c r="AI4" s="64" t="s">
+        <v>25</v>
+      </c>
+      <c r="AJ4" s="64" t="s">
         <v>35</v>
       </c>
-      <c r="W4" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="X4" s="63" t="s">
+      <c r="AK4" s="64" t="s">
+        <v>26</v>
+      </c>
+      <c r="AL4" s="64" t="s">
         <v>36</v>
       </c>
-      <c r="Y4" s="63" t="s">
-        <v>25</v>
-      </c>
-      <c r="Z4" s="63" t="s">
-        <v>25</v>
-      </c>
-      <c r="AA4" s="63" t="s">
+      <c r="AM4" s="64" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN4" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="AB4" s="63" t="s">
-        <v>37</v>
-      </c>
-      <c r="AC4" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="AD4" s="63" t="s">
-        <v>26</v>
-      </c>
-      <c r="AE4" s="63" t="s">
+      <c r="AO4" s="64" t="s">
+        <v>28</v>
+      </c>
+      <c r="AP4" s="64" t="s">
         <v>38</v>
       </c>
-      <c r="AF4" s="63" t="s">
-        <v>38</v>
-      </c>
-      <c r="AG4" s="63" t="s">
-        <v>27</v>
-      </c>
-      <c r="AH4" s="63" t="s">
-        <v>39</v>
-      </c>
-      <c r="AI4" s="64" t="s">
-        <v>28</v>
-      </c>
-      <c r="AJ4" s="64" t="s">
-        <v>40</v>
-      </c>
-      <c r="AK4" s="64" t="s">
-        <v>29</v>
-      </c>
-      <c r="AL4" s="64" t="s">
-        <v>41</v>
-      </c>
-      <c r="AM4" s="64" t="s">
-        <v>30</v>
-      </c>
-      <c r="AN4" s="64" t="s">
-        <v>42</v>
-      </c>
-      <c r="AO4" s="64" t="s">
-        <v>31</v>
-      </c>
-      <c r="AP4" s="64" t="s">
-        <v>43</v>
-      </c>
     </row>
-    <row r="5" spans="1:42" s="62" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:42" s="62" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A5" s="65" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B5" s="59" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C5" s="59" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D5" s="59" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="F5" s="59" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G5" s="60">
         <v>20</v>
@@ -1411,7 +1420,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A6" s="35">
         <v>45383</v>
       </c>
@@ -1545,7 +1554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A7" s="36">
         <v>45384</v>
       </c>
@@ -1679,7 +1688,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A8" s="36">
         <v>45385</v>
       </c>
@@ -1813,7 +1822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A9" s="36">
         <v>45386</v>
       </c>
@@ -1947,7 +1956,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A10" s="36">
         <v>45387</v>
       </c>
@@ -2081,7 +2090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A11" s="36">
         <v>45388</v>
       </c>
@@ -2215,7 +2224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A12" s="36">
         <v>45389</v>
       </c>
@@ -2349,7 +2358,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A13" s="36">
         <v>45390</v>
       </c>
@@ -2483,7 +2492,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A14" s="36">
         <v>45391</v>
       </c>
@@ -2617,7 +2626,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A15" s="36">
         <v>45392</v>
       </c>
@@ -2751,7 +2760,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A16" s="36">
         <v>45393</v>
       </c>
@@ -2885,7 +2894,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A17" s="36">
         <v>45394</v>
       </c>
@@ -3019,7 +3028,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A18" s="36">
         <v>45395</v>
       </c>
@@ -3153,7 +3162,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A19" s="36">
         <v>45396</v>
       </c>
@@ -3287,7 +3296,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A20" s="36">
         <v>45397</v>
       </c>
@@ -3421,7 +3430,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A21" s="36">
         <v>45398</v>
       </c>
@@ -3555,7 +3564,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A22" s="36">
         <v>45399</v>
       </c>
@@ -3689,7 +3698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A23" s="36">
         <v>45400</v>
       </c>
@@ -3823,7 +3832,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A24" s="36">
         <v>45401</v>
       </c>
@@ -3957,7 +3966,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A25" s="36">
         <v>45402</v>
       </c>
@@ -4091,7 +4100,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A26" s="36">
         <v>45403</v>
       </c>
@@ -4225,7 +4234,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A27" s="36">
         <v>45404</v>
       </c>
@@ -4359,7 +4368,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A28" s="36">
         <v>45405</v>
       </c>
@@ -4493,7 +4502,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A29" s="36">
         <v>45406</v>
       </c>
@@ -4627,7 +4636,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A30" s="36">
         <v>45407</v>
       </c>
@@ -4761,7 +4770,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A31" s="36">
         <v>45408</v>
       </c>
@@ -4895,7 +4904,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A32" s="36">
         <v>45409</v>
       </c>
@@ -5029,7 +5038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A33" s="36">
         <v>45410</v>
       </c>
@@ -5163,7 +5172,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="34" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A34" s="36">
         <v>45411</v>
       </c>
@@ -5297,7 +5306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A35" s="37">
         <v>45412</v>
       </c>
@@ -5431,7 +5440,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A36" s="35">
         <v>45413</v>
       </c>
@@ -5565,7 +5574,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A37" s="36">
         <v>45414</v>
       </c>
@@ -5699,7 +5708,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A38" s="36">
         <v>45415</v>
       </c>
@@ -5833,7 +5842,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A39" s="36">
         <v>45416</v>
       </c>
@@ -5967,7 +5976,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A40" s="36">
         <v>45417</v>
       </c>
@@ -6101,7 +6110,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A41" s="36">
         <v>45418</v>
       </c>
@@ -6235,7 +6244,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A42" s="36">
         <v>45419</v>
       </c>
@@ -6369,7 +6378,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A43" s="36">
         <v>45420</v>
       </c>
@@ -6503,7 +6512,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A44" s="36">
         <v>45421</v>
       </c>
@@ -6637,7 +6646,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="45" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A45" s="36">
         <v>45422</v>
       </c>
@@ -6771,7 +6780,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A46" s="36">
         <v>45423</v>
       </c>
@@ -6905,7 +6914,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A47" s="36">
         <v>45424</v>
       </c>
@@ -7039,7 +7048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A48" s="36">
         <v>45425</v>
       </c>
@@ -7173,7 +7182,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A49" s="36">
         <v>45426</v>
       </c>
@@ -7307,7 +7316,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A50" s="36">
         <v>45427</v>
       </c>
@@ -7441,7 +7450,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A51" s="36">
         <v>45428</v>
       </c>
@@ -7575,7 +7584,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A52" s="36">
         <v>45429</v>
       </c>
@@ -7709,7 +7718,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A53" s="36">
         <v>45430</v>
       </c>
@@ -7843,7 +7852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A54" s="36">
         <v>45431</v>
       </c>
@@ -7977,7 +7986,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A55" s="36">
         <v>45432</v>
       </c>
@@ -8111,7 +8120,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A56" s="36">
         <v>45433</v>
       </c>
@@ -8245,7 +8254,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A57" s="36">
         <v>45434</v>
       </c>
@@ -8379,7 +8388,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A58" s="36">
         <v>45435</v>
       </c>
@@ -8513,7 +8522,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A59" s="36">
         <v>45436</v>
       </c>
@@ -8647,7 +8656,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A60" s="36">
         <v>45437</v>
       </c>
@@ -8781,7 +8790,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A61" s="36">
         <v>45438</v>
       </c>
@@ -8915,7 +8924,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A62" s="36">
         <v>45439</v>
       </c>
@@ -9049,7 +9058,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A63" s="36">
         <v>45440</v>
       </c>
@@ -9183,7 +9192,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A64" s="36">
         <v>45441</v>
       </c>
@@ -9317,7 +9326,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A65" s="36">
         <v>45442</v>
       </c>
@@ -9451,7 +9460,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A66" s="37">
         <v>45443</v>
       </c>
@@ -9585,7 +9594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A67" s="35">
         <v>45444</v>
       </c>
@@ -9719,7 +9728,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A68" s="36">
         <v>45445</v>
       </c>
@@ -9853,7 +9862,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A69" s="36">
         <v>45446</v>
       </c>
@@ -9987,7 +9996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A70" s="36">
         <v>45447</v>
       </c>
@@ -10121,7 +10130,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A71" s="36">
         <v>45448</v>
       </c>
@@ -10255,7 +10264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A72" s="36">
         <v>45449</v>
       </c>
@@ -10389,7 +10398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A73" s="36">
         <v>45450</v>
       </c>
@@ -10523,7 +10532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A74" s="36">
         <v>45451</v>
       </c>
@@ -10657,7 +10666,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A75" s="36">
         <v>45452</v>
       </c>
@@ -10791,7 +10800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A76" s="36">
         <v>45453</v>
       </c>
@@ -10925,7 +10934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A77" s="36">
         <v>45454</v>
       </c>
@@ -11059,7 +11068,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:42" s="7" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A78" s="36">
         <v>45455</v>
       </c>
@@ -11193,7 +11202,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="79" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A79" s="36">
         <v>45456</v>
       </c>
@@ -11327,7 +11336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A80" s="36">
         <v>45457</v>
       </c>
@@ -11461,7 +11470,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A81" s="36">
         <v>45458</v>
       </c>
@@ -11595,7 +11604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="82" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A82" s="36">
         <v>45459</v>
       </c>
@@ -11729,7 +11738,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A83" s="36">
         <v>45460</v>
       </c>
@@ -11863,7 +11872,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A84" s="36">
         <v>45461</v>
       </c>
@@ -11997,7 +12006,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A85" s="36">
         <v>45462</v>
       </c>
@@ -12131,7 +12140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A86" s="36">
         <v>45463</v>
       </c>
@@ -12265,7 +12274,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A87" s="36">
         <v>45464</v>
       </c>
@@ -12399,7 +12408,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A88" s="36">
         <v>45465</v>
       </c>
@@ -12533,7 +12542,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A89" s="36">
         <v>45466</v>
       </c>
@@ -12667,7 +12676,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A90" s="36">
         <v>45467</v>
       </c>
@@ -12801,7 +12810,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A91" s="36">
         <v>45468</v>
       </c>
@@ -12935,7 +12944,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="92" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A92" s="36">
         <v>45469</v>
       </c>
@@ -13069,7 +13078,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A93" s="36">
         <v>45470</v>
       </c>
@@ -13203,7 +13212,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A94" s="36">
         <v>45471</v>
       </c>
@@ -13337,7 +13346,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:42" x14ac:dyDescent="0.45">
       <c r="A95" s="36">
         <v>45472</v>
       </c>
@@ -13471,7 +13480,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="96" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:42" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A96" s="37">
         <v>45473</v>
       </c>
@@ -13605,7 +13614,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A97" s="35">
         <v>45474</v>
       </c>
@@ -13739,7 +13748,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A98" s="36">
         <v>45475</v>
       </c>
@@ -13873,7 +13882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A99" s="36">
         <v>45476</v>
       </c>
@@ -14007,7 +14016,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A100" s="36">
         <v>45477</v>
       </c>
@@ -14141,7 +14150,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A101" s="36">
         <v>45478</v>
       </c>
@@ -14275,7 +14284,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A102" s="36">
         <v>45479</v>
       </c>
@@ -14409,7 +14418,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="103" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A103" s="36">
         <v>45480</v>
       </c>
@@ -14543,7 +14552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A104" s="36">
         <v>45481</v>
       </c>
@@ -14677,7 +14686,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A105" s="36">
         <v>45482</v>
       </c>
@@ -14811,7 +14820,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="106" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A106" s="36">
         <v>45483</v>
       </c>
@@ -14945,7 +14954,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="107" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A107" s="36">
         <v>45484</v>
       </c>
@@ -15079,7 +15088,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="108" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A108" s="36">
         <v>45485</v>
       </c>
@@ -15213,7 +15222,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="109" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A109" s="36">
         <v>45486</v>
       </c>
@@ -15347,7 +15356,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A110" s="36">
         <v>45487</v>
       </c>
@@ -15481,7 +15490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="111" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A111" s="36">
         <v>45488</v>
       </c>
@@ -15615,7 +15624,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="112" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A112" s="36">
         <v>45489</v>
       </c>
@@ -15749,7 +15758,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A113" s="36">
         <v>45490</v>
       </c>
@@ -15883,7 +15892,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A114" s="36">
         <v>45491</v>
       </c>
@@ -16017,7 +16026,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A115" s="36">
         <v>45492</v>
       </c>
@@ -16151,7 +16160,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A116" s="36">
         <v>45493</v>
       </c>
@@ -16285,7 +16294,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A117" s="36">
         <v>45494</v>
       </c>
@@ -16419,7 +16428,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A118" s="36">
         <v>45495</v>
       </c>
@@ -16553,7 +16562,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A119" s="36">
         <v>45496</v>
       </c>
@@ -16687,7 +16696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="120" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A120" s="36">
         <v>45497</v>
       </c>
@@ -16821,7 +16830,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A121" s="36">
         <v>45498</v>
       </c>
@@ -16955,7 +16964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A122" s="36">
         <v>45499</v>
       </c>
@@ -17089,7 +17098,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="123" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A123" s="36">
         <v>45500</v>
       </c>
@@ -17223,7 +17232,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A124" s="36">
         <v>45501</v>
       </c>
@@ -17357,7 +17366,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A125" s="36">
         <v>45502</v>
       </c>
@@ -17491,7 +17500,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="126" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A126" s="36">
         <v>45503</v>
       </c>
@@ -17625,7 +17634,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A127" s="37">
         <v>45504</v>
       </c>
@@ -17759,7 +17768,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A128" s="35">
         <v>45505</v>
       </c>
@@ -17893,7 +17902,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A129" s="36">
         <v>45506</v>
       </c>
@@ -18027,7 +18036,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A130" s="36">
         <v>45507</v>
       </c>
@@ -18161,7 +18170,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A131" s="36">
         <v>45508</v>
       </c>
@@ -18295,7 +18304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="132" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A132" s="36">
         <v>45509</v>
       </c>
@@ -18429,7 +18438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A133" s="36">
         <v>45510</v>
       </c>
@@ -18563,7 +18572,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A134" s="36">
         <v>45511</v>
       </c>
@@ -18697,7 +18706,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A135" s="36">
         <v>45512</v>
       </c>
@@ -18831,7 +18840,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="136" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A136" s="36">
         <v>45513</v>
       </c>
@@ -18965,7 +18974,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="137" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A137" s="36">
         <v>45514</v>
       </c>
@@ -19099,7 +19108,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="138" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A138" s="36">
         <v>45515</v>
       </c>
@@ -19233,7 +19242,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="139" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A139" s="36">
         <v>45516</v>
       </c>
@@ -19367,7 +19376,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="140" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A140" s="36">
         <v>45517</v>
       </c>
@@ -19501,7 +19510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A141" s="36">
         <v>45518</v>
       </c>
@@ -19635,7 +19644,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="142" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A142" s="36">
         <v>45519</v>
       </c>
@@ -19769,7 +19778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="143" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A143" s="36">
         <v>45520</v>
       </c>
@@ -19903,7 +19912,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="144" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A144" s="36">
         <v>45521</v>
       </c>
@@ -20037,7 +20046,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="145" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A145" s="36">
         <v>45522</v>
       </c>
@@ -20171,7 +20180,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A146" s="36">
         <v>45523</v>
       </c>
@@ -20305,7 +20314,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A147" s="36">
         <v>45524</v>
       </c>
@@ -20439,7 +20448,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A148" s="36">
         <v>45525</v>
       </c>
@@ -20573,7 +20582,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A149" s="36">
         <v>45526</v>
       </c>
@@ -20707,7 +20716,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A150" s="36">
         <v>45527</v>
       </c>
@@ -20841,7 +20850,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A151" s="36">
         <v>45528</v>
       </c>
@@ -20975,7 +20984,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A152" s="36">
         <v>45529</v>
       </c>
@@ -21109,7 +21118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A153" s="36">
         <v>45530</v>
       </c>
@@ -21243,7 +21252,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A154" s="36">
         <v>45531</v>
       </c>
@@ -21377,7 +21386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="155" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A155" s="36">
         <v>45532</v>
       </c>
@@ -21511,7 +21520,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="156" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A156" s="36">
         <v>45533</v>
       </c>
@@ -21645,7 +21654,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="157" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A157" s="36">
         <v>45534</v>
       </c>
@@ -21779,7 +21788,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="158" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A158" s="37">
         <v>45535</v>
       </c>
@@ -21913,7 +21922,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A159" s="35">
         <v>45536</v>
       </c>
@@ -22047,7 +22056,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="160" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A160" s="36">
         <v>45537</v>
       </c>
@@ -22181,7 +22190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A161" s="36">
         <v>45538</v>
       </c>
@@ -22315,7 +22324,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A162" s="36">
         <v>45539</v>
       </c>
@@ -22449,7 +22458,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="163" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A163" s="36">
         <v>45540</v>
       </c>
@@ -22583,7 +22592,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="164" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A164" s="36">
         <v>45541</v>
       </c>
@@ -22717,7 +22726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="165" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A165" s="36">
         <v>45542</v>
       </c>
@@ -22851,7 +22860,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="166" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A166" s="36">
         <v>45543</v>
       </c>
@@ -22985,7 +22994,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="167" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A167" s="36">
         <v>45544</v>
       </c>
@@ -23119,7 +23128,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="168" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A168" s="36">
         <v>45545</v>
       </c>
@@ -23253,7 +23262,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="169" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A169" s="36">
         <v>45546</v>
       </c>
@@ -23387,7 +23396,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A170" s="36">
         <v>45547</v>
       </c>
@@ -23521,7 +23530,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="171" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A171" s="36">
         <v>45548</v>
       </c>
@@ -23655,7 +23664,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A172" s="36">
         <v>45549</v>
       </c>
@@ -23789,7 +23798,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="173" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A173" s="36">
         <v>45550</v>
       </c>
@@ -23923,7 +23932,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="174" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A174" s="36">
         <v>45551</v>
       </c>
@@ -24057,7 +24066,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A175" s="36">
         <v>45552</v>
       </c>
@@ -24191,7 +24200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A176" s="36">
         <v>45553</v>
       </c>
@@ -24325,7 +24334,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="177" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A177" s="36">
         <v>45554</v>
       </c>
@@ -24458,7 +24467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A178" s="36">
         <v>45555</v>
       </c>
@@ -24591,7 +24600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="179" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A179" s="36">
         <v>45556</v>
       </c>
@@ -24724,7 +24733,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="180" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A180" s="36">
         <v>45557</v>
       </c>
@@ -24857,7 +24866,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A181" s="36">
         <v>45558</v>
       </c>
@@ -24990,7 +24999,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="182" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A182" s="36">
         <v>45559</v>
       </c>
@@ -25123,7 +25132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="183" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A183" s="36">
         <v>45560</v>
       </c>
@@ -25256,7 +25265,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="184" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A184" s="36">
         <v>45561</v>
       </c>
@@ -25389,7 +25398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A185" s="36">
         <v>45562</v>
       </c>
@@ -25522,7 +25531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A186" s="36">
         <v>45563</v>
       </c>
@@ -25655,7 +25664,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A187" s="36">
         <v>45564</v>
       </c>
@@ -25788,7 +25797,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A188" s="37">
         <v>45565</v>
       </c>
@@ -25921,7 +25930,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A189" s="35">
         <v>45566</v>
       </c>
@@ -26055,7 +26064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A190" s="36">
         <v>45567</v>
       </c>
@@ -26189,7 +26198,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A191" s="36">
         <v>45568</v>
       </c>
@@ -26323,7 +26332,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A192" s="36">
         <v>45569</v>
       </c>
@@ -26457,7 +26466,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A193" s="36">
         <v>45570</v>
       </c>
@@ -26591,7 +26600,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="194" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A194" s="36">
         <v>45571</v>
       </c>
@@ -26725,7 +26734,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="195" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A195" s="36">
         <v>45572</v>
       </c>
@@ -26859,7 +26868,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A196" s="36">
         <v>45573</v>
       </c>
@@ -26993,7 +27002,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A197" s="36">
         <v>45574</v>
       </c>
@@ -27127,7 +27136,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A198" s="36">
         <v>45575</v>
       </c>
@@ -27261,7 +27270,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="199" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A199" s="36">
         <v>45576</v>
       </c>
@@ -27395,7 +27404,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="200" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A200" s="36">
         <v>45577</v>
       </c>
@@ -27529,7 +27538,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="201" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A201" s="36">
         <v>45578</v>
       </c>
@@ -27663,7 +27672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="202" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A202" s="36">
         <v>45579</v>
       </c>
@@ -27797,7 +27806,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A203" s="36">
         <v>45580</v>
       </c>
@@ -27931,7 +27940,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A204" s="36">
         <v>45581</v>
       </c>
@@ -28065,7 +28074,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A205" s="36">
         <v>45582</v>
       </c>
@@ -28199,7 +28208,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A206" s="36">
         <v>45583</v>
       </c>
@@ -28333,7 +28342,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A207" s="36">
         <v>45584</v>
       </c>
@@ -28467,7 +28476,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A208" s="36">
         <v>45585</v>
       </c>
@@ -28601,7 +28610,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A209" s="36">
         <v>45586</v>
       </c>
@@ -28735,7 +28744,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A210" s="36">
         <v>45587</v>
       </c>
@@ -28869,7 +28878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A211" s="36">
         <v>45588</v>
       </c>
@@ -29003,7 +29012,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A212" s="36">
         <v>45589</v>
       </c>
@@ -29137,7 +29146,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A213" s="36">
         <v>45590</v>
       </c>
@@ -29271,7 +29280,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A214" s="36">
         <v>45591</v>
       </c>
@@ -29405,7 +29414,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A215" s="36">
         <v>45592</v>
       </c>
@@ -29539,7 +29548,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A216" s="36">
         <v>45593</v>
       </c>
@@ -29673,7 +29682,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A217" s="36">
         <v>45594</v>
       </c>
@@ -29807,7 +29816,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A218" s="36">
         <v>45595</v>
       </c>
@@ -29941,7 +29950,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A219" s="37">
         <v>45596</v>
       </c>
@@ -30075,7 +30084,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="220" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A220" s="35">
         <v>45597</v>
       </c>
@@ -30209,7 +30218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="221" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A221" s="36">
         <v>45598</v>
       </c>
@@ -30343,7 +30352,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="222" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A222" s="36">
         <v>45599</v>
       </c>
@@ -30477,7 +30486,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="1:42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:42" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A223" s="36">
         <v>45600</v>
       </c>
@@ -30611,7 +30620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A224" s="36">
         <v>45601</v>
       </c>
@@ -30745,7 +30754,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="225" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A225" s="36">
         <v>45602</v>
       </c>
@@ -30879,7 +30888,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A226" s="36">
         <v>45603</v>
       </c>
@@ -31013,7 +31022,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="227" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A227" s="36">
         <v>45604</v>
       </c>
@@ -31147,7 +31156,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="228" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A228" s="36">
         <v>45605</v>
       </c>
@@ -31281,7 +31290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="229" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A229" s="36">
         <v>45606</v>
       </c>
@@ -31415,7 +31424,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="230" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A230" s="36">
         <v>45607</v>
       </c>
@@ -31549,7 +31558,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="231" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A231" s="36">
         <v>45608</v>
       </c>
@@ -31683,7 +31692,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="232" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A232" s="36">
         <v>45609</v>
       </c>
@@ -31817,7 +31826,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="233" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A233" s="36">
         <v>45610</v>
       </c>
@@ -31951,7 +31960,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A234" s="36">
         <v>45611</v>
       </c>
@@ -32085,7 +32094,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="235" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A235" s="36">
         <v>45612</v>
       </c>
@@ -32219,7 +32228,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="236" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A236" s="36">
         <v>45613</v>
       </c>
@@ -32353,7 +32362,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="237" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A237" s="36">
         <v>45614</v>
       </c>
@@ -32487,7 +32496,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A238" s="36">
         <v>45615</v>
       </c>
@@ -32621,7 +32630,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="239" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A239" s="36">
         <v>45616</v>
       </c>
@@ -32755,7 +32764,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="240" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A240" s="36">
         <v>45617</v>
       </c>
@@ -32889,7 +32898,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A241" s="36">
         <v>45618</v>
       </c>
@@ -33023,7 +33032,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A242" s="36">
         <v>45619</v>
       </c>
@@ -33157,7 +33166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="243" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A243" s="36">
         <v>45620</v>
       </c>
@@ -33291,7 +33300,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A244" s="36">
         <v>45621</v>
       </c>
@@ -33425,7 +33434,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="245" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A245" s="36">
         <v>45622</v>
       </c>
@@ -33559,7 +33568,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A246" s="36">
         <v>45623</v>
       </c>
@@ -33693,7 +33702,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="247" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A247" s="36">
         <v>45624</v>
       </c>
@@ -33827,7 +33836,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="248" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A248" s="36">
         <v>45625</v>
       </c>
@@ -33961,7 +33970,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="249" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A249" s="37">
         <v>45626</v>
       </c>
@@ -34095,7 +34104,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="250" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A250" s="35">
         <v>45627</v>
       </c>
@@ -34229,7 +34238,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="251" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A251" s="36">
         <v>45628</v>
       </c>
@@ -34363,7 +34372,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="252" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A252" s="36">
         <v>45629</v>
       </c>
@@ -34497,7 +34506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A253" s="36">
         <v>45630</v>
       </c>
@@ -34631,7 +34640,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="254" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A254" s="36">
         <v>45631</v>
       </c>
@@ -34765,7 +34774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A255" s="36">
         <v>45632</v>
       </c>
@@ -34899,7 +34908,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="256" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A256" s="36">
         <v>45633</v>
       </c>
@@ -35033,7 +35042,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="257" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A257" s="36">
         <v>45634</v>
       </c>
@@ -35167,7 +35176,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="258" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A258" s="36">
         <v>45635</v>
       </c>
@@ -35301,7 +35310,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="259" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A259" s="36">
         <v>45636</v>
       </c>
@@ -35435,7 +35444,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="260" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A260" s="36">
         <v>45637</v>
       </c>
@@ -35569,7 +35578,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A261" s="36">
         <v>45638</v>
       </c>
@@ -35703,7 +35712,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A262" s="36">
         <v>45639</v>
       </c>
@@ -35837,7 +35846,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="263" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A263" s="36">
         <v>45640</v>
       </c>
@@ -35971,7 +35980,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A264" s="36">
         <v>45641</v>
       </c>
@@ -36105,7 +36114,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="265" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A265" s="36">
         <v>45642</v>
       </c>
@@ -36239,7 +36248,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="266" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A266" s="36">
         <v>45643</v>
       </c>
@@ -36373,7 +36382,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="267" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A267" s="36">
         <v>45644</v>
       </c>
@@ -36507,7 +36516,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="268" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A268" s="36">
         <v>45645</v>
       </c>
@@ -36641,7 +36650,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="269" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A269" s="36">
         <v>45646</v>
       </c>
@@ -36775,7 +36784,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="270" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A270" s="36">
         <v>45647</v>
       </c>
@@ -36909,7 +36918,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="271" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A271" s="36">
         <v>45648</v>
       </c>
@@ -37043,7 +37052,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="272" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A272" s="36">
         <v>45649</v>
       </c>
@@ -37177,7 +37186,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="273" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A273" s="36">
         <v>45650</v>
       </c>
@@ -37311,7 +37320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="274" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A274" s="36">
         <v>45651</v>
       </c>
@@ -37445,7 +37454,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="275" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A275" s="36">
         <v>45652</v>
       </c>
@@ -37579,7 +37588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="276" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A276" s="36">
         <v>45653</v>
       </c>
@@ -37713,7 +37722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="277" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A277" s="36">
         <v>45654</v>
       </c>
@@ -37847,7 +37856,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="278" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A278" s="36">
         <v>45655</v>
       </c>
@@ -37981,7 +37990,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="279" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A279" s="36">
         <v>45656</v>
       </c>
@@ -38115,7 +38124,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="280" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A280" s="37">
         <v>45657</v>
       </c>
@@ -38249,7 +38258,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="281" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A281" s="35">
         <v>45658</v>
       </c>
@@ -38383,7 +38392,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="282" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A282" s="36">
         <v>45659</v>
       </c>
@@ -38517,7 +38526,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="283" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A283" s="36">
         <v>45660</v>
       </c>
@@ -38651,7 +38660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="284" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A284" s="36">
         <v>45661</v>
       </c>
@@ -38785,7 +38794,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="285" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A285" s="36">
         <v>45662</v>
       </c>
@@ -38919,7 +38928,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="286" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A286" s="36">
         <v>45663</v>
       </c>
@@ -39053,7 +39062,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="287" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A287" s="36">
         <v>45664</v>
       </c>
@@ -39187,7 +39196,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="288" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A288" s="36">
         <v>45665</v>
       </c>
@@ -39321,7 +39330,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="289" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A289" s="36">
         <v>45666</v>
       </c>
@@ -39455,7 +39464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="290" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A290" s="36">
         <v>45667</v>
       </c>
@@ -39589,7 +39598,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="291" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A291" s="36">
         <v>45668</v>
       </c>
@@ -39723,7 +39732,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="292" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A292" s="36">
         <v>45669</v>
       </c>
@@ -39857,7 +39866,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="293" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A293" s="36">
         <v>45670</v>
       </c>
@@ -39991,7 +40000,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="294" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A294" s="36">
         <v>45671</v>
       </c>
@@ -40125,7 +40134,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="295" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A295" s="36">
         <v>45672</v>
       </c>
@@ -40259,7 +40268,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="296" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A296" s="36">
         <v>45673</v>
       </c>
@@ -40393,7 +40402,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="297" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A297" s="36">
         <v>45674</v>
       </c>
@@ -40527,7 +40536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="298" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A298" s="36">
         <v>45675</v>
       </c>
@@ -40661,7 +40670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="299" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A299" s="36">
         <v>45676</v>
       </c>
@@ -40795,7 +40804,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="300" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A300" s="36">
         <v>45677</v>
       </c>
@@ -40929,7 +40938,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="301" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A301" s="36">
         <v>45678</v>
       </c>
@@ -41063,7 +41072,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="302" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A302" s="36">
         <v>45679</v>
       </c>
@@ -41197,7 +41206,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="303" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A303" s="36">
         <v>45680</v>
       </c>
@@ -41331,7 +41340,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="304" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A304" s="36">
         <v>45681</v>
       </c>
@@ -41465,7 +41474,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="305" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A305" s="36">
         <v>45682</v>
       </c>
@@ -41599,7 +41608,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="306" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A306" s="36">
         <v>45683</v>
       </c>
@@ -41733,7 +41742,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="307" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A307" s="36">
         <v>45684</v>
       </c>
@@ -41867,7 +41876,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="308" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A308" s="36">
         <v>45685</v>
       </c>
@@ -42001,7 +42010,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="309" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A309" s="36">
         <v>45686</v>
       </c>
@@ -42135,7 +42144,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="310" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A310" s="36">
         <v>45687</v>
       </c>
@@ -42269,7 +42278,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="311" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A311" s="37">
         <v>45688</v>
       </c>
@@ -42403,7 +42412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="312" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A312" s="35">
         <v>45689</v>
       </c>
@@ -42537,7 +42546,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="313" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A313" s="36">
         <v>45690</v>
       </c>
@@ -42671,7 +42680,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="314" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A314" s="36">
         <v>45691</v>
       </c>
@@ -42805,7 +42814,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="315" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A315" s="36">
         <v>45692</v>
       </c>
@@ -42939,7 +42948,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="316" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A316" s="36">
         <v>45693</v>
       </c>
@@ -43073,7 +43082,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="317" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A317" s="36">
         <v>45694</v>
       </c>
@@ -43207,7 +43216,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="318" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A318" s="36">
         <v>45695</v>
       </c>
@@ -43341,7 +43350,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="319" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A319" s="36">
         <v>45696</v>
       </c>
@@ -43475,7 +43484,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="320" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A320" s="36">
         <v>45697</v>
       </c>
@@ -43609,7 +43618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="321" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A321" s="36">
         <v>45698</v>
       </c>
@@ -43743,7 +43752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="322" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A322" s="36">
         <v>45699</v>
       </c>
@@ -43877,7 +43886,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A323" s="36">
         <v>45700</v>
       </c>
@@ -44011,7 +44020,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="324" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A324" s="36">
         <v>45701</v>
       </c>
@@ -44145,7 +44154,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="325" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A325" s="36">
         <v>45702</v>
       </c>
@@ -44279,7 +44288,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="326" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A326" s="36">
         <v>45703</v>
       </c>
@@ -44413,7 +44422,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="327" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A327" s="36">
         <v>45704</v>
       </c>
@@ -44547,7 +44556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="328" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A328" s="36">
         <v>45705</v>
       </c>
@@ -44681,7 +44690,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="329" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A329" s="36">
         <v>45706</v>
       </c>
@@ -44815,7 +44824,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="330" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A330" s="36">
         <v>45707</v>
       </c>
@@ -44949,7 +44958,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="331" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A331" s="36">
         <v>45708</v>
       </c>
@@ -45083,7 +45092,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="332" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A332" s="36">
         <v>45709</v>
       </c>
@@ -45217,7 +45226,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="333" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A333" s="36">
         <v>45710</v>
       </c>
@@ -45351,7 +45360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="334" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A334" s="36">
         <v>45711</v>
       </c>
@@ -45485,7 +45494,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="335" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A335" s="36">
         <v>45712</v>
       </c>
@@ -45619,7 +45628,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A336" s="36">
         <v>45713</v>
       </c>
@@ -45753,7 +45762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="337" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A337" s="36">
         <v>45714</v>
       </c>
@@ -45887,7 +45896,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="338" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A338" s="36">
         <v>45715</v>
       </c>
@@ -46021,7 +46030,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="339" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="339" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A339" s="37">
         <v>45716</v>
       </c>
@@ -46155,7 +46164,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="340" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A340" s="46">
         <v>45717</v>
       </c>
@@ -46289,7 +46298,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="341" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A341" s="36">
         <v>45718</v>
       </c>
@@ -46423,7 +46432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="342" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A342" s="36">
         <v>45719</v>
       </c>
@@ -46557,7 +46566,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="343" spans="1:42" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:42" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A343" s="36">
         <v>45720</v>
       </c>
@@ -46691,7 +46700,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="344" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A344" s="36">
         <v>45721</v>
       </c>
@@ -46825,7 +46834,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="345" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A345" s="36">
         <v>45722</v>
       </c>
@@ -46959,7 +46968,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="346" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A346" s="36">
         <v>45723</v>
       </c>
@@ -47093,7 +47102,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="347" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A347" s="36">
         <v>45724</v>
       </c>
@@ -47227,7 +47236,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="348" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A348" s="36">
         <v>45725</v>
       </c>
@@ -47361,7 +47370,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="349" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A349" s="36">
         <v>45726</v>
       </c>
@@ -47495,7 +47504,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="350" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A350" s="36">
         <v>45727</v>
       </c>
@@ -47629,7 +47638,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="351" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A351" s="36">
         <v>45728</v>
       </c>
@@ -47763,7 +47772,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="352" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:42" s="7" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A352" s="36">
         <v>45729</v>
       </c>
@@ -47897,7 +47906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="353" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A353" s="36">
         <v>45730</v>
       </c>
@@ -48031,7 +48040,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="354" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A354" s="36">
         <v>45731</v>
       </c>
@@ -48165,7 +48174,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="355" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A355" s="36">
         <v>45732</v>
       </c>
@@ -48299,7 +48308,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="356" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A356" s="36">
         <v>45733</v>
       </c>
@@ -48433,7 +48442,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="357" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A357" s="36">
         <v>45734</v>
       </c>
@@ -48567,7 +48576,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="358" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A358" s="36">
         <v>45735</v>
       </c>
@@ -48701,7 +48710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="359" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A359" s="36">
         <v>45736</v>
       </c>
@@ -48835,7 +48844,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="360" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A360" s="36">
         <v>45737</v>
       </c>
@@ -48969,7 +48978,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="361" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A361" s="36">
         <v>45738</v>
       </c>
@@ -49103,7 +49112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="362" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A362" s="36">
         <v>45739</v>
       </c>
@@ -49237,7 +49246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="363" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A363" s="36">
         <v>45740</v>
       </c>
@@ -49371,7 +49380,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="364" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A364" s="36">
         <v>45741</v>
       </c>
@@ -49505,7 +49514,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="365" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A365" s="36">
         <v>45742</v>
       </c>
@@ -49639,7 +49648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="366" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A366" s="36">
         <v>45743</v>
       </c>
@@ -49773,7 +49782,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="367" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A367" s="36">
         <v>45744</v>
       </c>
@@ -49907,7 +49916,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="368" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A368" s="36">
         <v>45745</v>
       </c>
@@ -50041,7 +50050,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="369" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A369" s="36">
         <v>45746</v>
       </c>
@@ -50175,7 +50184,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="370" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="370" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A370" s="37">
         <v>45747</v>
       </c>
@@ -50309,7 +50318,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="371" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A371" s="46">
         <v>45748</v>
       </c>
@@ -50443,7 +50452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="372" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A372" s="36">
         <v>45749</v>
       </c>
@@ -50577,7 +50586,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="373" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A373" s="46">
         <v>45750</v>
       </c>
@@ -50711,7 +50720,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="374" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A374" s="36">
         <v>45751</v>
       </c>
@@ -50845,7 +50854,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="375" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A375" s="46">
         <v>45752</v>
       </c>
@@ -50979,7 +50988,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="376" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A376" s="36">
         <v>45753</v>
       </c>
@@ -51113,7 +51122,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="377" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A377" s="46">
         <v>45754</v>
       </c>
@@ -51247,7 +51256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="378" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A378" s="36">
         <v>45755</v>
       </c>
@@ -51381,7 +51390,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="379" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A379" s="46">
         <v>45756</v>
       </c>
@@ -51515,7 +51524,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="380" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A380" s="36">
         <v>45757</v>
       </c>
@@ -51649,7 +51658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="381" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A381" s="46">
         <v>45758</v>
       </c>
@@ -51783,7 +51792,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="382" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A382" s="36">
         <v>45759</v>
       </c>
@@ -51917,7 +51926,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="383" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A383" s="46">
         <v>45760</v>
       </c>
@@ -52051,7 +52060,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="384" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A384" s="36">
         <v>45761</v>
       </c>
@@ -52185,7 +52194,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="385" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A385" s="46">
         <v>45762</v>
       </c>
@@ -52319,7 +52328,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="386" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A386" s="36">
         <v>45763</v>
       </c>
@@ -52453,7 +52462,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="387" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A387" s="46">
         <v>45764</v>
       </c>
@@ -52587,7 +52596,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="388" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A388" s="36">
         <v>45765</v>
       </c>
@@ -52721,7 +52730,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="389" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A389" s="46">
         <v>45766</v>
       </c>
@@ -52855,7 +52864,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="390" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A390" s="36">
         <v>45767</v>
       </c>
@@ -52989,7 +52998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="391" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A391" s="46">
         <v>45768</v>
       </c>
@@ -53123,7 +53132,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="392" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A392" s="36">
         <v>45769</v>
       </c>
@@ -53257,7 +53266,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="393" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A393" s="46">
         <v>45770</v>
       </c>
@@ -53391,7 +53400,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="394" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A394" s="36">
         <v>45771</v>
       </c>
@@ -53525,7 +53534,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="395" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A395" s="46">
         <v>45772</v>
       </c>
@@ -53659,7 +53668,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="396" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A396" s="36">
         <v>45773</v>
       </c>
@@ -53793,7 +53802,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="397" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A397" s="46">
         <v>45774</v>
       </c>
@@ -53927,7 +53936,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="398" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A398" s="36">
         <v>45775</v>
       </c>
@@ -54061,7 +54070,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="399" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A399" s="46">
         <v>45776</v>
       </c>
@@ -54195,7 +54204,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="400" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="400" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A400" s="37">
         <v>45777</v>
       </c>
@@ -54329,7 +54338,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="401" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A401" s="46">
         <v>45778</v>
       </c>
@@ -54463,7 +54472,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="402" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A402" s="36">
         <v>45779</v>
       </c>
@@ -54597,7 +54606,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="403" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A403" s="46">
         <v>45780</v>
       </c>
@@ -54731,7 +54740,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="404" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A404" s="36">
         <v>45781</v>
       </c>
@@ -54865,7 +54874,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="405" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A405" s="46">
         <v>45782</v>
       </c>
@@ -54999,7 +55008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="406" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A406" s="36">
         <v>45783</v>
       </c>
@@ -55133,7 +55142,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="407" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A407" s="46">
         <v>45784</v>
       </c>
@@ -55267,7 +55276,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="408" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A408" s="36">
         <v>45785</v>
       </c>
@@ -55401,7 +55410,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="409" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A409" s="46">
         <v>45786</v>
       </c>
@@ -55535,7 +55544,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="410" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A410" s="36">
         <v>45787</v>
       </c>
@@ -55669,7 +55678,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="411" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A411" s="46">
         <v>45788</v>
       </c>
@@ -55803,7 +55812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="412" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A412" s="36">
         <v>45789</v>
       </c>
@@ -55937,7 +55946,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="413" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A413" s="46">
         <v>45790</v>
       </c>
@@ -56071,7 +56080,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="414" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A414" s="36">
         <v>45791</v>
       </c>
@@ -56205,7 +56214,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="415" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A415" s="46">
         <v>45792</v>
       </c>
@@ -56339,7 +56348,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="416" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A416" s="36">
         <v>45793</v>
       </c>
@@ -56473,7 +56482,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="417" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A417" s="46">
         <v>45794</v>
       </c>
@@ -56607,7 +56616,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="418" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A418" s="36">
         <v>45795</v>
       </c>
@@ -56741,7 +56750,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="419" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A419" s="46">
         <v>45796</v>
       </c>
@@ -56875,7 +56884,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="420" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A420" s="36">
         <v>45797</v>
       </c>
@@ -57009,7 +57018,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="421" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A421" s="46">
         <v>45798</v>
       </c>
@@ -57143,7 +57152,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="422" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A422" s="36">
         <v>45799</v>
       </c>
@@ -57277,7 +57286,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="423" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A423" s="46">
         <v>45800</v>
       </c>
@@ -57411,7 +57420,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="424" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A424" s="36">
         <v>45801</v>
       </c>
@@ -57545,7 +57554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="425" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A425" s="46">
         <v>45802</v>
       </c>
@@ -57679,7 +57688,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="426" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A426" s="36">
         <v>45803</v>
       </c>
@@ -57813,7 +57822,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="427" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A427" s="46">
         <v>45804</v>
       </c>
@@ -57947,7 +57956,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="428" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A428" s="36">
         <v>45805</v>
       </c>
@@ -58081,7 +58090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="429" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A429" s="46">
         <v>45806</v>
       </c>
@@ -58215,7 +58224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="430" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A430" s="36">
         <v>45807</v>
       </c>
@@ -58349,7 +58358,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="431" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="431" spans="1:42" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A431" s="37">
         <v>45808</v>
       </c>
@@ -58496,6 +58505,28 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c9c6ccd3-328d-4385-98b9-897146d5bd1f">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0d6975ae-f676-438f-a851-2189cd451402" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7891F75A989B644A5B94CB860E198CF" ma:contentTypeVersion="21" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7ca8a1c2ae0cb43ebb6fa39eb6e8c867">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="c9c6ccd3-328d-4385-98b9-897146d5bd1f" xmlns:ns3="0d6975ae-f676-438f-a851-2189cd451402" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="40ca73d8a9fb501e987503ba4dec0552" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -58773,36 +58804,42 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="c9c6ccd3-328d-4385-98b9-897146d5bd1f">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0d6975ae-f676-438f-a851-2189cd451402" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A286FA3-621D-4029-BA21-69A3CB6400C4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B1F4F3C-80E5-4802-954E-3D9F6C54327A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2B1F4F3C-80E5-4802-954E-3D9F6C54327A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA3A364-1979-4C2F-B1B5-C9DFF6E53C8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c9c6ccd3-328d-4385-98b9-897146d5bd1f"/>
+    <ds:schemaRef ds:uri="0d6975ae-f676-438f-a851-2189cd451402"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CFA3A364-1979-4C2F-B1B5-C9DFF6E53C8F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A286FA3-621D-4029-BA21-69A3CB6400C4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="c9c6ccd3-328d-4385-98b9-897146d5bd1f"/>
+    <ds:schemaRef ds:uri="0d6975ae-f676-438f-a851-2189cd451402"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>